<commit_message>
cycle time test results
</commit_message>
<xml_diff>
--- a/test/Cycle_Time_Test.xlsx
+++ b/test/Cycle_Time_Test.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sean\Desktop\P2_Battery_Disassembly\test\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57440028-A55A-4207-8514-ACEB3263E4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,28 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="5">
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>✓</t>
+  </si>
+  <si>
+    <t>Warmup run</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -37,7 +63,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -45,12 +71,103 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +447,110 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="8">
+        <v>23.67</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5">
+        <v>21.29</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5">
+        <v>21.26</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5">
+        <v>21.21</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>4</v>
+      </c>
+      <c r="B8" s="10">
+        <v>21.23</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="6"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
+        <v>5</v>
+      </c>
+      <c r="B9" s="11">
+        <v>21.23</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="9"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added test results for the accuracy and repeatability for the rigid gripper
</commit_message>
<xml_diff>
--- a/test/Cycle_Time_Test.xlsx
+++ b/test/Cycle_Time_Test.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sean\Desktop\P2_Battery_Disassembly\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rasmuslykke/Desktop/P2_Battery_Disassembly/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57440028-A55A-4207-8514-ACEB3263E4E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477BDB5C-B4DD-2D46-AA74-2168527E9FC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
   <si>
     <t>Time</t>
   </si>
@@ -40,6 +51,15 @@
   </si>
   <si>
     <t>Warmup run</t>
+  </si>
+  <si>
+    <t>Time (s)</t>
+  </si>
+  <si>
+    <t>avg time (s)</t>
+  </si>
+  <si>
+    <t>std deviation (s)</t>
   </si>
 </sst>
 </file>
@@ -155,19 +175,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,13 +465,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -466,22 +483,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="7">
         <v>23.67</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="9" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C2" s="7"/>
+      <c r="D2" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="2" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>2</v>
@@ -490,65 +507,88 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>21.29</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>2</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>21.26</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="5"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>3</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7">
         <v>21.21</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>4</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8">
         <v>21.23</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="7">
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="6">
         <v>5</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="7">
         <v>21.23</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" s="9"/>
+      <c r="C9" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="8"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="3">
+        <f>AVERAGE(B5:B9)</f>
+        <v>21.244</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="8">
+        <f>23-B11</f>
+        <v>1.7560000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D18">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>